<commit_message>
Rebuild the synthetic sample report
</commit_message>
<xml_diff>
--- a/docs/sample/break_report_SYNTHETIC.xlsx
+++ b/docs/sample/break_report_SYNTHETIC.xlsx
@@ -15,12 +15,14 @@
     <sheet name="Restatements" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Data Quality" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Holdings" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Answers" sheetId="8" state="visible" r:id="rId10"/>
-    <sheet name="About" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Approved Prices" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Answers" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="About" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="true" localSheetId="7" name="_xlnm._FilterDatabase" vbProcedure="false">'Approved Prices'!$A$1:$F$13</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Cleared!$A$1:$M$12</definedName>
-    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Data Quality'!$A$1:$E$4</definedName>
+    <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Data Quality'!$A$1:$E$6</definedName>
     <definedName function="false" hidden="true" localSheetId="6" name="_xlnm._FilterDatabase" vbProcedure="false">Holdings!$A$1:$M$2</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'New Today'!$A$1:$K$3</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Open Breaks'!$A$1:$U$20</definedName>
@@ -36,12 +38,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="241">
   <si>
     <t xml:space="preserve">JSE price reconciliation: break report</t>
   </si>
   <si>
-    <t xml:space="preserve">As of 2026-09-11. Generated 2026-09-30 10:30 SAST. Every count below is a formula over the tab named beside it.</t>
+    <t xml:space="preserve">As of 2026-09-11. Generated 2026-09-30 10:57 SAST. Every count below is a formula over the tab named beside it.</t>
   </si>
   <si>
     <t xml:space="preserve">Breaks between sources</t>
@@ -146,6 +148,15 @@
     <t xml:space="preserve">Gross difference (R)</t>
   </si>
   <si>
+    <t xml:space="preserve">  of which errors (R)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  of which timing differences (R)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Positions that could not be valued</t>
+  </si>
+  <si>
     <t xml:space="preserve">Recon</t>
   </si>
   <si>
@@ -428,12 +439,21 @@
     <t xml:space="preserve">synthetic_a</t>
   </si>
   <si>
+    <t xml:space="preserve">Missing price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No price on a trading day</t>
+  </si>
+  <si>
     <t xml:space="preserve">Frozen price</t>
   </si>
   <si>
     <t xml:space="preserve">R49.73 unchanged for 6 sessions</t>
   </si>
   <si>
+    <t xml:space="preserve">synthetic_b</t>
+  </si>
+  <si>
     <t xml:space="preserve">Price on closed day</t>
   </si>
   <si>
@@ -443,9 +463,6 @@
     <t xml:space="preserve">1 prices on National Women's Day (observed), 1 with volume</t>
   </si>
   <si>
-    <t xml:space="preserve">synthetic_b</t>
-  </si>
-  <si>
     <t xml:space="preserve">Statement lines</t>
   </si>
   <si>
@@ -476,100 +493,133 @@
     <t xml:space="preserve">No broker statement loaded</t>
   </si>
   <si>
+    <t xml:space="preserve">Price to use (R)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For 2026-09-11; exceptions first</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TO_VERIFY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The sources disagree and the break has no resolution yet: confirm before use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APPROVED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary source, passed every check</t>
+  </si>
+  <si>
     <t xml:space="preserve">Can synthetic_a be trusted to value a fund of JSE shares?</t>
   </si>
   <si>
+    <t xml:space="preserve">Evidence: snapshot 2026-09-11, 347 closing prices for 12 securities, 2026-08-03 to 2026-09-11.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Are the prices right?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   No. Of all 347 stored prices, 2026-08-03 to 2026-09-11, each as the latest snapshot holding it has it, 1 (0.288%) were about 100x wrong, on 1 days: 2026-08-20 (1 securities).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Separately, 2 day-on-day moves of 15% or more that the median share did not share (by 10% or more). These are not errors in themselves: each needs checking against company news before the price is used. The feed's adjusted close did not adjust 2 of them, so it cannot tell a corporate action from an error.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. What would those errors have cost?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   For any fund: a price 100x too small understates the fund by 99% of that holding's weight, so a single holding above 0.51% of the fund breaches the 0.5% ASISA tolerance on its own.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Worst day for a Top 40 fund, 2026-08-20: 1,188bp (11.88% of NAV), 23.8x the tolerance, from SYC. Basis: SYNTHETIC weights at 2025-12-31.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Illustrative, equal-weighted across all 12 securities priced on 2026-08-20: 825bp (8.25%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   A unit check or a day-on-day movement check catches errors this large. The cost is what a fund valued from the raw feed, without those controls, would have shown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Is every trading day there?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Yes, all 29 trading days in the JSE calendar are present.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Does the vendor rewrite history, or publish late?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Between snapshots 2026-09-10 and 2026-09-11, fetched 24 hours apart: 1 of 323 prices were rewritten, and 12 appeared only in the later snapshot. One pair of snapshots so far; re-measured with every new one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   2026-09-10 was published late. The ASISA standard allows the last available price only after checking it is fair and reasonable. Used unchecked, the previous day's prices would have misstated a Top 40 fund by +174bp (3.5x the tolerance; SYNTHETIC weights at 2025-12-31), or an equal-weighted fund of 12 securities by +79bp. Whether the delay matters depends on the fund's valuation point and publication deadline.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Is the list of securities still accurate?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   None of the 12 codes has been renamed or delisted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Are any prices suspiciously frozen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   1 times a price stayed identical for 5+ sessions. Longest: SYE, 6 sessions to 2026-08-19. 1 of the 1 had no volume after the first day, the mark of a suspension or a feed filling gaps; the others traded at an unchanged price, common for thinly traded shares. Each needs checking against a trading suspension.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Do independent sources agree?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   synthetic_a vs synthetic_b (12 securities, to 2026-09-11): 329 of 347 closes agree (94.8%); breaks: SCALE 9, VAL 6, STALE 2, CAL 1, UNIT 1. Volumes differed on 0% of matched days.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. When sources disagree, does it get fixed, and how fast?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   synthetic_a_vs_synthetic_b: 30 disagreements tracked. 11 cleared within 2 trading days (timing differences), 0 took longer, and 19 are still open. Those that cleared took 1.0 trading days on average.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Analyst resolutions on the open breaks: no resolution yet 19 (config/break_notes.yaml).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   17 of the open breaks were already there in the first comparison of that share, so their age counts from the price date, not from when they were found.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Oldest open: SYJ on 2026-08-10, 24 trading days after that price date.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Largest open: SYI on 2026-09-08, -99.4% apart (SCALE), which would cost a Top 40 fund 4.97% of NAV if the wrong price were used.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9. Does the broker statement agree with the internal book?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   No broker statement loaded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10. Which price should the fund use today, and why?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   For 2026-09-11, using synthetic_a first, then synthetic_b, then the previous close: 11 approved, 1 to verify, 0 from synthetic_b, 0 carried forward.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   TO_VERIFY, 1: The sources disagree and the break has no resolution yet: confirm before use (SYI).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Each share's price, source and reason are on the Approved Prices tab of the report.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can synthetic_b be trusted to value a fund of JSE shares?</t>
+  </si>
+  <si>
     <t xml:space="preserve">Evidence: snapshot 2026-09-11, 348 closing prices for 12 securities, 2026-08-03 to 2026-09-11.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Are the prices right?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   No. Of all 348 stored prices, 2026-08-03 to 2026-09-11, each as the latest snapshot holding it has it, 1 (0.287%) were about 100x wrong, on 1 days: 2026-08-20 (1 securities).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Separately, 2 day-on-day moves of 15% or more that the median share did not share (by 10% or more). These are not errors in themselves: each needs checking against company news before the price is used. The feed's adjusted close did not adjust 2 of them, so it cannot tell a corporate action from an error.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. What would those errors have cost?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   For any fund: a price 100x too small understates the fund by 99% of that holding's weight, so a single holding above 0.51% of the fund breaches the 0.5% ASISA tolerance on its own.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Worst day for a Top 40 fund, 2026-08-20: 1,188bp (11.88% of NAV), 23.8x the tolerance, from SYC. Basis: SYNTHETIC weights at 2025-12-31.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Illustrative, equal-weighted across all 12 securities priced on 2026-08-20: 825bp (8.25%).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   A unit check or a day-on-day movement check catches errors this large. The cost is what a fund valued from the raw feed, without those controls, would have shown.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Is every trading day there?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Yes, all 29 trading days in the JSE calendar are present.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Does the vendor rewrite history, or publish late?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Between snapshots 2026-09-10 and 2026-09-11, fetched 24 hours apart: 1 of 324 prices were rewritten, and 12 appeared only in the later snapshot. One pair of snapshots so far; re-measured with every new one.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   2026-09-10 was published late. The ASISA standard allows the last available price only after checking it is fair and reasonable. Used unchecked, the previous day's prices would have misstated a Top 40 fund by +174bp (3.5x the tolerance; SYNTHETIC weights at 2025-12-31), or an equal-weighted fund of 12 securities by +79bp. Whether the delay matters depends on the fund's valuation point and publication deadline.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Is the list of securities still accurate?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   None of the 12 codes has been renamed or delisted.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Are any prices suspiciously frozen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   1 times a price stayed identical for 5+ sessions. Longest: SYE, 6 sessions to 2026-08-19. Each needs checking against a trading suspension.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Do independent sources agree?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   synthetic_a vs synthetic_b (12 securities, to 2026-09-11): 330 of 348 closes agree (94.8%); breaks: SCALE 9, VAL 6, STALE 2, CAL 1, UNIT 1. Volumes differed on 0% of matched days.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8. When sources disagree, does it get fixed, and how fast?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   synthetic_a_vs_synthetic_b: 30 disagreements tracked. 11 cleared within 2 trading days (timing differences), 0 took longer, and 19 are still open. Those that cleared took 1.0 trading days on average.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Analyst resolutions on the open breaks: no resolution yet 19 (config/break_notes.yaml).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   17 of the open breaks were already there in the first comparison of that share, so their age counts from the price date, not from when they were found.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Oldest open: SYJ on 2026-08-10, 24 trading days after that price date.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Largest open: SYI on 2026-09-08, -99.4% apart (SCALE), which would cost a Top 40 fund 4.97% of NAV if the wrong price were used.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9. Does the broker statement agree with the internal book?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   No broker statement loaded.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Can synthetic_b be trusted to value a fund of JSE shares?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence: snapshot 2026-09-11, 349 closing prices for 12 securities, 2026-08-03 to 2026-09-11.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   No unit errors in all 349 stored prices, 2026-08-03 to 2026-09-11, each as the latest snapshot holding it has it.</t>
+    <t xml:space="preserve">   No unit errors in all 348 stored prices, 2026-08-03 to 2026-09-11, each as the latest snapshot holding it has it.</t>
   </si>
   <si>
     <t xml:space="preserve">   Separately, 3 day-on-day moves of 15% or more that the median share did not share (by 10% or more). These are not errors in themselves: each needs checking against company news before the price is used. The feed's adjusted close did not adjust 3 of them, so it cannot tell a corporate action from an error.</t>
@@ -578,7 +628,7 @@
     <t xml:space="preserve">   Nothing to cost.</t>
   </si>
   <si>
-    <t xml:space="preserve">   Between snapshots 2026-09-10 and 2026-09-11, fetched 24 hours apart: 0 of 337 prices were rewritten, and 0 appeared only in the later snapshot. One pair of snapshots so far; re-measured with every new one.</t>
+    <t xml:space="preserve">   Between snapshots 2026-09-10 and 2026-09-11, fetched 24 hours apart: 0 of 336 prices were rewritten, and 0 appeared only in the later snapshot. One pair of snapshots so far; re-measured with every new one.</t>
   </si>
   <si>
     <t xml:space="preserve">   None frozen for 5+ sessions.</t>
@@ -593,7 +643,7 @@
     <t xml:space="preserve">Generated</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-30 10:30 SAST</t>
+    <t xml:space="preserve">2026-09-30 10:57 SAST</t>
   </si>
   <si>
     <t xml:space="preserve">Latest synthetic_a snapshot</t>
@@ -705,6 +755,9 @@
   </si>
   <si>
     <t xml:space="preserve">A value break where one side's price has not moved for 5 or more sessions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The sides are more than 50% apart but not about 100x: a different instrument or scale</t>
   </si>
   <si>
     <t xml:space="preserve">A break that cleared within 2 trading days of first being seen</t>
@@ -722,7 +775,7 @@
     <numFmt numFmtId="168" formatCode="\R#,##0.00;&quot;(R&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -768,6 +821,26 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
@@ -784,14 +857,14 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="11"/>
+      <sz val="12"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -807,7 +880,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -888,7 +961,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -896,20 +969,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -921,11 +994,19 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="9">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF1F3864"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF8D7D7"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -955,8 +1036,30 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill>
+          <bgColor rgb="FFF8D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFCEBC7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF808080"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCEBC7"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -982,12 +1085,12 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFCEBC7"/>
+      <rgbColor rgb="FFD9E1F2"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD9E1F2"/>
+      <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -1003,15 +1106,15 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFF8D7D7"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF4F81BD"/>
+      <rgbColor rgb="FF878787"/>
       <rgbColor rgb="FF1F3864"/>
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
@@ -1025,8 +1128,313 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Open breaks by age</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4f81bd"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Summary!$A$6:$A$9</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>  open 0-1 days</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>  open 2-5 days</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>  open 6-20 days</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>  open 21+ days</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Summary!$B$6:$B$9</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="81865006"/>
+        <c:axId val="38421569"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="81865006"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="38421569"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="38421569"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr b="1" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:rPr>
+                  <a:t>Breaks</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="81865006"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>160920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>525600</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>34560</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="0" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="7337520" y="571680"/>
+        <a:ext cx="4319640" cy="2159640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1046,6 +1454,14 @@
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
@@ -1229,7 +1645,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1475,7 +1891,7 @@
       </c>
       <c r="B23" s="5" t="n">
         <f aca="false">COUNTIFS('Data Quality'!$A:$A,"Missing price")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>24</v>
@@ -1570,6 +1986,300 @@
       </c>
       <c r="C31" s="2" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" s="8" t="n">
+        <f aca="false">SUMPRODUCT(ABS(Holdings!$L$2:$L$2000)*(Holdings!$B$2:$B$2000&lt;&gt;"MATCH")*(Holdings!$B$2:$B$2000&lt;&gt;"SETTLE"))</f>
+        <v>0</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="8" t="n">
+        <f aca="false">SUMPRODUCT(ABS(Holdings!$L$2:$L$2000)*(Holdings!$B$2:$B$2000="SETTLE"))</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B34" s="5" t="n">
+        <f aca="false">SUMPRODUCT((Holdings!$B$2:$B$2000&lt;&gt;"")*(Holdings!$L$2:$L$2000=""))</f>
+        <v>0</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2"/>
+      <c r="B19" s="14"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="B20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B28" s="14" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -1610,81 +2320,81 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="O1" s="9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="P1" s="9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="Q1" s="9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="R1" s="9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="S1" s="9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="T1" s="9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="U1" s="9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E2" s="10" t="n">
         <v>46244</v>
@@ -1703,7 +2413,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="K2" s="8"/>
       <c r="L2" s="8" t="n">
@@ -1712,7 +2422,7 @@
       <c r="M2" s="8"/>
       <c r="N2" s="7"/>
       <c r="O2" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
@@ -1720,7 +2430,7 @@
         <v>24</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T2" s="7" t="n">
         <v>0.04</v>
@@ -1732,16 +2442,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E3" s="10" t="n">
         <v>46254</v>
@@ -1760,7 +2470,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="K3" s="8" t="n">
         <v>0.301812</v>
@@ -1775,7 +2485,7 @@
         <v>99</v>
       </c>
       <c r="O3" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
@@ -1783,7 +2493,7 @@
         <v>16</v>
       </c>
       <c r="S3" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T3" s="7" t="n">
         <v>0.12</v>
@@ -1795,16 +2505,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>46273</v>
@@ -1823,7 +2533,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K4" s="8" t="n">
         <v>79.8234</v>
@@ -1838,7 +2548,7 @@
         <v>-0.993750003131914</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="P4" s="2"/>
       <c r="Q4" s="2"/>
@@ -1846,7 +2556,7 @@
         <v>3</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T4" s="7" t="n">
         <v>0.05</v>
@@ -1858,16 +2568,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>46268</v>
@@ -1886,7 +2596,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K5" s="8" t="n">
         <v>80.6258</v>
@@ -1901,7 +2611,7 @@
         <v>-0.993750003100745</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
@@ -1909,7 +2619,7 @@
         <v>6</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T5" s="7" t="n">
         <v>0.05</v>
@@ -1921,16 +2631,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>46274</v>
@@ -1949,7 +2659,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K6" s="8" t="n">
         <v>79.7437</v>
@@ -1964,7 +2674,7 @@
         <v>-0.993750001567522</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
@@ -1972,7 +2682,7 @@
         <v>2</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T6" s="7" t="n">
         <v>0.05</v>
@@ -1984,16 +2694,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>46269</v>
@@ -2012,7 +2722,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K7" s="8" t="n">
         <v>79.8205</v>
@@ -2027,7 +2737,7 @@
         <v>-0.993750001566014</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="P7" s="2"/>
       <c r="Q7" s="2"/>
@@ -2035,7 +2745,7 @@
         <v>5</v>
       </c>
       <c r="S7" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T7" s="7" t="n">
         <v>0.05</v>
@@ -2047,16 +2757,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>46266</v>
@@ -2075,7 +2785,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K8" s="8" t="n">
         <v>89.5808</v>
@@ -2090,7 +2800,7 @@
         <v>-0.99375</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
@@ -2098,7 +2808,7 @@
         <v>8</v>
       </c>
       <c r="S8" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T8" s="7" t="n">
         <v>0.05</v>
@@ -2110,16 +2820,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>46267</v>
@@ -2138,7 +2848,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K9" s="8" t="n">
         <v>89.9094</v>
@@ -2153,7 +2863,7 @@
         <v>-0.993749997219423</v>
       </c>
       <c r="O9" s="2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="P9" s="2"/>
       <c r="Q9" s="2"/>
@@ -2161,7 +2871,7 @@
         <v>7</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T9" s="7" t="n">
         <v>0.05</v>
@@ -2173,16 +2883,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>46276</v>
@@ -2201,7 +2911,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K10" s="8" t="n">
         <v>78.8494</v>
@@ -2216,7 +2926,7 @@
         <v>-0.993749996829399</v>
       </c>
       <c r="O10" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="P10" s="2"/>
       <c r="Q10" s="2"/>
@@ -2224,7 +2934,7 @@
         <v>0</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T10" s="7" t="n">
         <v>0.05</v>
@@ -2236,16 +2946,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>46272</v>
@@ -2264,7 +2974,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K11" s="8" t="n">
         <v>79.5041</v>
@@ -2279,7 +2989,7 @@
         <v>-0.993749995283262</v>
       </c>
       <c r="O11" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="P11" s="2"/>
       <c r="Q11" s="2"/>
@@ -2287,7 +2997,7 @@
         <v>4</v>
       </c>
       <c r="S11" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T11" s="7" t="n">
         <v>0.05</v>
@@ -2299,16 +3009,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E12" s="10" t="n">
         <v>46275</v>
@@ -2327,7 +3037,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="K12" s="8" t="n">
         <v>79.2484</v>
@@ -2342,7 +3052,7 @@
         <v>-0.993749993690724</v>
       </c>
       <c r="O12" s="2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
@@ -2350,7 +3060,7 @@
         <v>1</v>
       </c>
       <c r="S12" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T12" s="7" t="n">
         <v>0.05</v>
@@ -2362,16 +3072,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>46266</v>
@@ -2390,7 +3100,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="K13" s="8" t="n">
         <v>20.6397</v>
@@ -2405,7 +3115,7 @@
         <v>-0.0196078431372548</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
@@ -2413,7 +3123,7 @@
         <v>8</v>
       </c>
       <c r="S13" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="T13" s="7" t="n">
         <v>0.15</v>
@@ -2425,16 +3135,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>46253</v>
@@ -2453,7 +3163,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="K14" s="8" t="n">
         <v>49.7292</v>
@@ -2468,7 +3178,7 @@
         <v>0.010637613313707</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="P14" s="2"/>
       <c r="Q14" s="2"/>
@@ -2476,7 +3186,7 @@
         <v>17</v>
       </c>
       <c r="S14" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T14" s="7" t="n">
         <v>0.08</v>
@@ -2488,16 +3198,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E15" s="10" t="n">
         <v>46261</v>
@@ -2516,7 +3226,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="K15" s="8" t="n">
         <v>69.7592</v>
@@ -2531,7 +3241,7 @@
         <v>0.00757606165208308</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="P15" s="2"/>
       <c r="Q15" s="2"/>
@@ -2539,7 +3249,7 @@
         <v>11</v>
       </c>
       <c r="S15" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T15" s="7" t="n">
         <v>0.07</v>
@@ -2551,16 +3261,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>46261</v>
@@ -2579,7 +3289,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="K16" s="8" t="n">
         <v>61.3274</v>
@@ -2594,7 +3304,7 @@
         <v>0.00606254300687796</v>
       </c>
       <c r="O16" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="P16" s="2"/>
       <c r="Q16" s="2"/>
@@ -2602,7 +3312,7 @@
         <v>11</v>
       </c>
       <c r="S16" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T16" s="7" t="n">
         <v>0.08</v>
@@ -2614,16 +3324,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>46261</v>
@@ -2642,7 +3352,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="K17" s="8" t="n">
         <v>78.4238</v>
@@ -2657,7 +3367,7 @@
         <v>-0.00356269397810353</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
@@ -2665,7 +3375,7 @@
         <v>11</v>
       </c>
       <c r="S17" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T17" s="7" t="n">
         <v>0.06</v>
@@ -2677,16 +3387,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E18" s="10" t="n">
         <v>46252</v>
@@ -2705,7 +3415,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="K18" s="8" t="n">
         <v>49.7292</v>
@@ -2720,7 +3430,7 @@
         <v>0.00226627414074622</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="P18" s="2"/>
       <c r="Q18" s="2"/>
@@ -2728,7 +3438,7 @@
         <v>18</v>
       </c>
       <c r="S18" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T18" s="7" t="n">
         <v>0.08</v>
@@ -2740,16 +3450,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>46248</v>
@@ -2768,7 +3478,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="K19" s="8" t="n">
         <v>49.7292</v>
@@ -2783,7 +3493,7 @@
         <v>0.00184800881574613</v>
       </c>
       <c r="O19" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="P19" s="2"/>
       <c r="Q19" s="2"/>
@@ -2791,7 +3501,7 @@
         <v>20</v>
       </c>
       <c r="S19" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T19" s="7" t="n">
         <v>0.08</v>
@@ -2803,16 +3513,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E20" s="10" t="n">
         <v>46247</v>
@@ -2831,7 +3541,7 @@
         <v>0-1 days</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="K20" s="8" t="n">
         <v>49.7292</v>
@@ -2846,7 +3556,7 @@
         <v>-0.00116631677163517</v>
       </c>
       <c r="O20" s="2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
@@ -2854,7 +3564,7 @@
         <v>21</v>
       </c>
       <c r="S20" s="2" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="T20" s="7" t="n">
         <v>0.08</v>
@@ -2866,6 +3576,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:U20"/>
+  <conditionalFormatting sqref="A2:U5000">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+      <formula>$J2="SCALE"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+      <formula>$J2="UNIT"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+      <formula>$I2="21+ days"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2898,54 +3619,54 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D2" s="10" t="n">
         <v>46266</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>20.6397</v>
@@ -2960,27 +3681,27 @@
         <v>-0.0196078431372548</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>46276</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>78.8494</v>
@@ -2995,10 +3716,10 @@
         <v>-0.993749996829399</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3035,54 +3756,54 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G1" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="H1" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>103</v>
-      </c>
       <c r="K1" s="9" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D2" s="10" t="n">
         <v>46275</v>
@@ -3097,29 +3818,29 @@
         <v>1</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D3" s="10" t="n">
         <v>46275</v>
@@ -3134,29 +3855,29 @@
         <v>1</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>46275</v>
@@ -3171,29 +3892,29 @@
         <v>1</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>46275</v>
@@ -3208,29 +3929,29 @@
         <v>1</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>46275</v>
@@ -3245,29 +3966,29 @@
         <v>1</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>46275</v>
@@ -3282,29 +4003,29 @@
         <v>1</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>46275</v>
@@ -3319,29 +4040,29 @@
         <v>1</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>46275</v>
@@ -3356,29 +4077,29 @@
         <v>1</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D10" s="10" t="n">
         <v>46275</v>
@@ -3393,29 +4114,29 @@
         <v>1</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D11" s="10" t="n">
         <v>46275</v>
@@ -3430,29 +4151,29 @@
         <v>1</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D12" s="10" t="n">
         <v>46275</v>
@@ -3467,16 +4188,16 @@
         <v>1</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="I12" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
@@ -3512,36 +4233,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B2" s="10" t="n">
         <v>46266</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="D2" s="8" t="n">
         <v>20.235</v>
@@ -3553,18 +4274,18 @@
         <v>0.404699999999998</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8" t="n">
@@ -3572,18 +4293,18 @@
       </c>
       <c r="F3" s="8"/>
       <c r="G3" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B4" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D4" s="8"/>
       <c r="E4" s="8" t="n">
@@ -3591,18 +4312,18 @@
       </c>
       <c r="F4" s="8"/>
       <c r="G4" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8" t="n">
@@ -3610,18 +4331,18 @@
       </c>
       <c r="F5" s="8"/>
       <c r="G5" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D6" s="8"/>
       <c r="E6" s="8" t="n">
@@ -3629,18 +4350,18 @@
       </c>
       <c r="F6" s="8"/>
       <c r="G6" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="8" t="n">
@@ -3648,18 +4369,18 @@
       </c>
       <c r="F7" s="8"/>
       <c r="G7" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8" t="n">
@@ -3667,18 +4388,18 @@
       </c>
       <c r="F8" s="8"/>
       <c r="G8" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="8" t="n">
@@ -3686,18 +4407,18 @@
       </c>
       <c r="F9" s="8"/>
       <c r="G9" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B10" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="8" t="n">
@@ -3705,18 +4426,18 @@
       </c>
       <c r="F10" s="8"/>
       <c r="G10" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B11" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D11" s="8"/>
       <c r="E11" s="8" t="n">
@@ -3724,18 +4445,18 @@
       </c>
       <c r="F11" s="8"/>
       <c r="G11" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B12" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D12" s="8"/>
       <c r="E12" s="8" t="n">
@@ -3743,18 +4464,18 @@
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B13" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D13" s="8"/>
       <c r="E13" s="8" t="n">
@@ -3762,18 +4483,18 @@
       </c>
       <c r="F13" s="8"/>
       <c r="G13" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>46275</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D14" s="8"/>
       <c r="E14" s="8" t="n">
@@ -3781,7 +4502,7 @@
       </c>
       <c r="F14" s="8"/>
       <c r="G14" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -3802,7 +4523,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -3814,74 +4535,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>46254</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>86</v>
+        <v>121</v>
       </c>
       <c r="C3" s="10" t="n">
-        <v>46253</v>
+        <v>46265</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>46253</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="B5" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>46265</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C6" s="10" t="n">
         <v>46244</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>135</v>
+      <c r="D6" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E4"/>
+  <autoFilter ref="A1:E6"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3913,48 +4668,48 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3987,294 +4742,289 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A57"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="90"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
-        <v>146</v>
+    <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
-        <v>147</v>
+      <c r="A2" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>78.8494</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13"/>
+      <c r="A3" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>8.4601</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
-        <v>148</v>
+      <c r="A4" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>18.413</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>150</v>
+      <c r="A5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>27.8788</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>48.253</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
-        <v>151</v>
+      <c r="A7" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>44.6065</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>152</v>
+      <c r="A8" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>55.5231</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>153</v>
+      <c r="A9" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>62.2997</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
-        <v>154</v>
+      <c r="A10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>68.934</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>155</v>
+      <c r="A11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>95.5223</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>1009.3901</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>156</v>
       </c>
+      <c r="F12" s="2" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>106.0873</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="13" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="13" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="13" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="13" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="13" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="13" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="13" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="13" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="13" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="13" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="13" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="13" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="13" t="s">
-        <v>174</v>
-      </c>
-    </row>
   </sheetData>
+  <autoFilter ref="A1:F13"/>
+  <conditionalFormatting sqref="A2:F5000">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+      <formula>$E2="FALLBACK"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+      <formula>OR($E2="TO_VERIFY",$E2="SECONDARY")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4282,6 +5032,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4290,237 +5041,331 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:A65"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="13" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="14" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="14" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="14" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="14" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="14" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="14" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="14" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="14" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="B1" s="13" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="B2" s="13" t="s">
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="B3" s="13" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="14" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="B4" s="13" t="s">
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="14" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="14" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="14" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="14" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="14" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="14" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="14" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="14" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="14" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="14" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="14" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="14" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="14" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="14" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="14" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="14" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="B5" s="13" t="s">
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="14" t="s">
         <v>190</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2"/>
-      <c r="B19" s="13"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
-        <v>211</v>
-      </c>
-      <c r="B20" s="13"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B24" s="13" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>